<commit_message>
Excel has agraph. V0.1
</commit_message>
<xml_diff>
--- a/XTEST.xlsx
+++ b/XTEST.xlsx
@@ -13,6 +13,17 @@
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -55,6 +66,250 @@
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$A$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>X</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$A$2:$A$19</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="18"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Y</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$2:$B$19</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="18"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>125</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>216</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>343</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>512</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>729</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1331</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1728</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>2197</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>2744</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3375</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>4096</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>4913</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>5832</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:marker val="1"/>
+        <c:axId val="147909632"/>
+        <c:axId val="115831552"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="147909632"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="115831552"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="115831552"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="147909632"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>581025</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="แผนภูมิ 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -342,9 +597,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A2:B19"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
     <row r="2" spans="1:2">
       <c r="A2">
         <v>1</v>
@@ -526,6 +789,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add a new graph in T01.
</commit_message>
<xml_diff>
--- a/XTEST.xlsx
+++ b/XTEST.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="120" windowWidth="14295" windowHeight="4620"/>
+    <workbookView xWindow="480" yWindow="120" windowWidth="14295" windowHeight="4620" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="2">
   <si>
     <t>X</t>
   </si>
@@ -233,24 +233,24 @@
           </c:val>
         </c:ser>
         <c:marker val="1"/>
-        <c:axId val="147909632"/>
-        <c:axId val="115831552"/>
+        <c:axId val="144325632"/>
+        <c:axId val="144339712"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="147909632"/>
+        <c:axId val="144325632"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="115831552"/>
+        <c:crossAx val="144339712"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="115831552"/>
+        <c:axId val="144339712"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -258,13 +258,225 @@
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="147909632"/>
+        <c:crossAx val="144325632"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75000000000000011" l="0.70000000000000007" r="0.70000000000000007" t="0.75000000000000011" header="0.30000000000000004" footer="0.30000000000000004"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Y</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet2!$A$2:$A$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>51</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>61</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>71</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>81</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>91</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>101</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>111</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>121</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>131</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>141</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>151</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>161</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>171</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>181</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$B$2:$B$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="19"/>
+                <c:pt idx="0">
+                  <c:v>0.8414709848078965</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.99999020655070348</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.83665563853605607</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.40403764532306502</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>-0.15862266880470899</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.67022917584337471</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>-0.96611777000839294</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.95105465325437466</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>-0.62988799427445386</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.10598751175115685</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.45202578717835057</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-0.86455144861060829</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.99881522472357953</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-0.81160338713670044</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.363171365373259</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.2021498814156536</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-0.70240778557737105</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.97659086794356575</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-0.93645140011764405</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls/>
+        <c:marker val="1"/>
+        <c:axId val="105012608"/>
+        <c:axId val="105043840"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="105012608"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="105043840"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="105043840"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9525">
+            <a:noFill/>
+          </a:ln>
+        </c:spPr>
+        <c:crossAx val="105012608"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
       <c:layout/>
     </c:legend>
     <c:plotVisOnly val="1"/>
@@ -281,20 +493,55 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>581025</xdr:colOff>
-      <xdr:row>1</xdr:row>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>161925</xdr:colOff>
+      <xdr:row>0</xdr:row>
       <xdr:rowOff>142875</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>276225</xdr:colOff>
-      <xdr:row>16</xdr:row>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>466725</xdr:colOff>
+      <xdr:row>15</xdr:row>
       <xdr:rowOff>28575</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="แผนภูมิ 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>76199</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>161924</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>352424</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>133349</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="แผนภูมิ 2"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -795,10 +1042,209 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <f>SIN(A2)</f>
+        <v>0.8414709848078965</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3">
+        <f>A2+10</f>
+        <v>11</v>
+      </c>
+      <c r="B3">
+        <f t="shared" ref="B3:B20" si="0">SIN(A3)</f>
+        <v>-0.99999020655070348</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4">
+        <f t="shared" ref="A4:A20" si="1">A3+10</f>
+        <v>21</v>
+      </c>
+      <c r="B4">
+        <f t="shared" si="0"/>
+        <v>0.83665563853605607</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5">
+        <f t="shared" si="1"/>
+        <v>31</v>
+      </c>
+      <c r="B5">
+        <f t="shared" si="0"/>
+        <v>-0.40403764532306502</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6">
+        <f t="shared" si="1"/>
+        <v>41</v>
+      </c>
+      <c r="B6">
+        <f t="shared" si="0"/>
+        <v>-0.15862266880470899</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7">
+        <f t="shared" si="1"/>
+        <v>51</v>
+      </c>
+      <c r="B7">
+        <f t="shared" si="0"/>
+        <v>0.67022917584337471</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8">
+        <f t="shared" si="1"/>
+        <v>61</v>
+      </c>
+      <c r="B8">
+        <f t="shared" si="0"/>
+        <v>-0.96611777000839294</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9">
+        <f t="shared" si="1"/>
+        <v>71</v>
+      </c>
+      <c r="B9">
+        <f t="shared" si="0"/>
+        <v>0.95105465325437466</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10">
+        <f t="shared" si="1"/>
+        <v>81</v>
+      </c>
+      <c r="B10">
+        <f t="shared" si="0"/>
+        <v>-0.62988799427445386</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11">
+        <f t="shared" si="1"/>
+        <v>91</v>
+      </c>
+      <c r="B11">
+        <f t="shared" si="0"/>
+        <v>0.10598751175115685</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12">
+        <f t="shared" si="1"/>
+        <v>101</v>
+      </c>
+      <c r="B12">
+        <f t="shared" si="0"/>
+        <v>0.45202578717835057</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13">
+        <f t="shared" si="1"/>
+        <v>111</v>
+      </c>
+      <c r="B13">
+        <f t="shared" si="0"/>
+        <v>-0.86455144861060829</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14">
+        <f t="shared" si="1"/>
+        <v>121</v>
+      </c>
+      <c r="B14">
+        <f t="shared" si="0"/>
+        <v>0.99881522472357953</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15">
+        <f t="shared" si="1"/>
+        <v>131</v>
+      </c>
+      <c r="B15">
+        <f t="shared" si="0"/>
+        <v>-0.81160338713670044</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16">
+        <f t="shared" si="1"/>
+        <v>141</v>
+      </c>
+      <c r="B16">
+        <f t="shared" si="0"/>
+        <v>0.363171365373259</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17">
+        <f t="shared" si="1"/>
+        <v>151</v>
+      </c>
+      <c r="B17">
+        <f t="shared" si="0"/>
+        <v>0.2021498814156536</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18">
+        <f t="shared" si="1"/>
+        <v>161</v>
+      </c>
+      <c r="B18">
+        <f t="shared" si="0"/>
+        <v>-0.70240778557737105</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19">
+        <f t="shared" si="1"/>
+        <v>171</v>
+      </c>
+      <c r="B19">
+        <f t="shared" si="0"/>
+        <v>0.97659086794356575</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20">
+        <f t="shared" si="1"/>
+        <v>181</v>
+      </c>
+      <c r="B20">
+        <f t="shared" si="0"/>
+        <v>-0.93645140011764405</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>